<commit_message>
Updated 0.9.0.lisp + SpreadsheetLisp.xlsx with BETWIXT? and BETWEEN? functions, and removed deprecated FIELDFUNCTION function from BUILTINS.F to fix BUILTINS dependents
</commit_message>
<xml_diff>
--- a/lisp/SpreadsheetLisp.xlsx
+++ b/lisp/SpreadsheetLisp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ragti\Documents\SpreadsheetInstitute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{022EB2EA-8770-4369-8F47-BFFBF5620084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D6E6CEEE-2217-4046-B814-4B7F08E850D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25800" windowHeight="21600" xr2:uid="{7DC06FD3-AF6C-4947-91D9-16174F9813A4}"/>
+    <workbookView xWindow="25800" yWindow="0" windowWidth="25800" windowHeight="21600" xr2:uid="{7DC06FD3-AF6C-4947-91D9-16174F9813A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,13 +34,15 @@
     <definedName name="ARITY">_xlfn.LAMBDA(_xlop._arg1,_xlop._arg2,_xlop._arg3,_xlop._arg4,_xlop._arg5,_xlop._arg6,_xlop._arg7,_xlop._arg8,_xlop._arg9,_xlop._arg10,_xlop._arg11,_xlop._arg12,_xlop._arg13,_xlop._arg14,_xlop._arg15,_xlop._arg16,_xlop._arg17,_xlop._arg18,_xlop._arg19,_xlop._arg20,_xlop._arg21,_xlop._arg22,_xlop._arg23,_xlop._arg24,_xlop._arg25,SUM(IS(_xlpm._arg1), IS(_xlpm._arg2), IS(_xlpm._arg3), IS(_xlpm._arg4), IS(_xlpm._arg5),IS(_xlpm._arg6), IS(_xlpm._arg7), IS(_xlpm._arg8), IS(_xlpm._arg9), IS(_xlpm._arg10),IS(_xlpm._arg11), IS(_xlpm._arg12), IS(_xlpm._arg13), IS(_xlpm._arg14), IS(_xlpm._arg15),IS(_xlpm._arg16), IS(_xlpm._arg17), IS(_xlpm._arg18), IS(_xlpm._arg19), IS(_xlpm._arg20),IS(_xlpm._arg21), IS(_xlpm._arg22), IS(_xlpm._arg23), IS(_xlpm._arg24), IS(_xlpm._arg25)))</definedName>
     <definedName name="ASSERT">_xlfn.LAMBDA(_xlpm.condition,_xlop.message,IF(_xlpm.condition,TRUE,DEFAULT(_xlpm.message,"Assertion failed")))</definedName>
     <definedName name="BEGINSWITH?">_xlfn.LAMBDA(_xlpm.text,_xlpm.beginning,_xlop.case_insensitive?,_xlfn.REGEXTEST(_xlpm.text,FORMAT("^{1}",_xlpm.beginning),DEFAULT(_xlpm.case_insensitive?,YES)))</definedName>
+    <definedName name="BETWEEN?">_xlfn.LAMBDA(_xlpm.number_to_check,_xlpm.lower_bound,_xlpm.upper_bound,AND(GTE?(_xlpm.number_to_check,_xlpm.lower_bound),LTE?(_xlpm.number_to_check,_xlpm.upper_bound)))</definedName>
+    <definedName name="BETWIXT?">_xlfn.LAMBDA(_xlpm.number_to_check,_xlpm.lower_bound,_xlpm.upper_bound,AND(GREATERTHAN?(_xlpm.number_to_check,_xlpm.lower_bound),LESSTHAN?(_xlpm.number_to_check,_xlpm.upper_bound)))</definedName>
     <definedName name="BUILTINS">_xlfn.LAMBDA(_xlfn.VSTACK(BUILTINS.A(),BUILTINS.B(),BUILTINS.C(),BUILTINS.D(),BUILTINS.E(),BUILTINS.F(),BUILTINS.G(),BUILTINS.H(),BUILTINS.I(),BUILTINS.K(),BUILTINS.L(),BUILTINS.M(),BUILTINS.N(),BUILTINS.O(),BUILTINS.P(),BUILTINS.Q(),BUILTINS.R(),BUILTINS.S(),BUILTINS.T(),BUILTINS.U(),BUILTINS.V(),BUILTINS.W(),BUILTINS.X(),BUILTINS.Y(),BUILTINS.Z()))</definedName>
     <definedName name="BUILTINS.A">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("ABS", _xleta.ABS),_xlfn.HSTACK("ACCRINT", _xleta.ACCRINT),_xlfn.HSTACK("ACCRINTM", _xleta.ACCRINTM),_xlfn.HSTACK("ACOS", _xleta.ACOS),_xlfn.HSTACK("ACOSH", _xleta.ACOSH),_xlfn.HSTACK("ACOT", _xleta.ACOT),_xlfn.HSTACK("ACOTH", _xleta.ACOTH),_xlfn.HSTACK("ADDRESS", _xleta.ADDRESS),_xlfn.HSTACK("AGGREGATE", _xleta.AGGREGATE),_xlfn.HSTACK("AMORDEGRC", _xleta.AMORDEGRC),_xlfn.HSTACK("AMORLINC", _xleta.AMORLINC),_xlfn.HSTACK("AND", _xleta.AND),_xlfn.HSTACK("ARABIC", _xleta.ARABIC),_xlfn.HSTACK("AREAS", _xleta.AREAS),_xlfn.HSTACK("ARRAYTOTEXT", _xleta.ARRAYTOTEXT),_xlfn.HSTACK("ASC", _xleta.ASC),_xlfn.HSTACK("ASIN", _xleta.ASIN),_xlfn.HSTACK("ASINH", _xleta.ASINH),_xlfn.HSTACK("ATAN", _xleta.ATAN),_xlfn.HSTACK("ATAN2", _xleta.ATAN2),_xlfn.HSTACK("ATANH", _xleta.ATANH),_xlfn.HSTACK("AVEDEV", _xleta.AVEDEV),_xlfn.HSTACK("AVERAGE", _xleta.AVERAGE),_xlfn.HSTACK("AVERAGEA", _xleta.AVERAGEA),_xlfn.HSTACK("AVERAGEIF", _xleta.AVERAGEIF),_xlfn.HSTACK("AVERAGEIFS", _xleta.AVERAGEIFS)))</definedName>
     <definedName name="BUILTINS.B">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("BAHTTEXT", _xleta.BAHTTEXT),_xlfn.HSTACK("BASE", _xleta.BASE),_xlfn.HSTACK("BESSELI", _xleta.BESSELI),_xlfn.HSTACK("BESSELJ", _xleta.BESSELJ),_xlfn.HSTACK("BESSELK", _xleta.BESSELK),_xlfn.HSTACK("BESSELY", _xleta.BESSELY),_xlfn.HSTACK("BETA.DIST", _xleta.BETA.DIST),_xlfn.HSTACK("BETADIST", _xleta.BETADIST),_xlfn.HSTACK("BETAINV", _xleta.BETAINV),_xlfn.HSTACK("BIN2DEC", _xleta.BIN2DEC),_xlfn.HSTACK("BIN2HEX", _xleta.BIN2HEX),_xlfn.HSTACK("BIN2OCT", _xleta.BIN2OCT),_xlfn.HSTACK("BINOM.DIST", _xleta.BINOM.DIST),_xlfn.HSTACK("BINOM.DIST.RANGE", _xleta.BINOM.DIST.RANGE),_xlfn.HSTACK("BINOM.INV", _xleta.BINOM.INV),_xlfn.HSTACK("BINOMDIST", _xleta.BINOMDIST),_xlfn.HSTACK("BITAND", _xleta.BITAND),_xlfn.HSTACK("BITLSHIFT", _xleta.BITLSHIFT),_xlfn.HSTACK("BITOR", _xleta.BITOR),_xlfn.HSTACK("BITRSHIFT", _xleta.BITRSHIFT),_xlfn.HSTACK("BITXOR", _xleta.BITXOR),_xlfn.HSTACK("BYCOL", _xleta.BYCOL),_xlfn.HSTACK("BYROW", _xleta.BYROW)))</definedName>
     <definedName name="BUILTINS.C">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("CEILING", _xleta.CEILING),_xlfn.HSTACK("CEILING.MATH", _xleta.CEILING.MATH),_xlfn.HSTACK("CEILING.PRECISE", _xleta.CEILING.PRECISE),_xlfn.HSTACK("CELL", _xleta.CELL),_xlfn.HSTACK("CHAR", _xleta.CHAR),_xlfn.HSTACK("CHIDIST", _xleta.CHIDIST),_xlfn.HSTACK("CHIINV", _xleta.CHIINV),_xlfn.HSTACK("CHISQ.DIST", _xleta.CHISQ.DIST),_xlfn.HSTACK("CHISQ.DIST.RT", _xleta.CHISQ.DIST.RT),_xlfn.HSTACK("CHISQ.INV", _xleta.CHISQ.INV),_xlfn.HSTACK("CHISQ.INV.RT", _xleta.CHISQ.INV.RT),_xlfn.HSTACK("CHISQ.TEST", _xleta.CHISQ.TEST),_xlfn.HSTACK("CHITEST", _xleta.CHITEST),_xlfn.HSTACK("CHOOSE", _xleta.CHOOSE),_xlfn.HSTACK("CHOOSECOLS", _xleta.CHOOSECOLS),_xlfn.HSTACK("CHOOSEROWS", _xleta.CHOOSEROWS),_xlfn.HSTACK("CLEAN", _xleta.CLEAN),_xlfn.HSTACK("CODE", _xleta.CODE),_xlfn.HSTACK("COLUMN", _xleta.COLUMN),_xlfn.HSTACK("COLUMNS", _xleta.COLUMNS),_xlfn.HSTACK("COMBIN", _xleta.COMBIN),_xlfn.HSTACK("COMBINA", _xleta.COMBINA),_xlfn.HSTACK("COMPLEX", _xleta.COMPLEX),_xlfn.HSTACK("CONCAT", _xleta.CONCAT),_xlfn.HSTACK("CONCATENATE", _xleta.CONCATENATE),_xlfn.HSTACK("CONFIDENCE", _xleta.CONFIDENCE),_xlfn.HSTACK("CONFIDENCE.NORM", _xleta.CONFIDENCE.NORM),_xlfn.HSTACK("CONFIDENCE.T", _xleta.CONFIDENCE.T),_xlfn.HSTACK("CONVERT", _xleta.CONVERT),_xlfn.HSTACK("CORREL", _xleta.CORREL),_xlfn.HSTACK("COS", _xleta.COS),_xlfn.HSTACK("COSH", _xleta.COSH),_xlfn.HSTACK("COT", _xleta.COT),_xlfn.HSTACK("COTH", _xleta.COTH),_xlfn.HSTACK("COUNT", _xleta.COUNT),_xlfn.HSTACK("COUNTA", _xleta.COUNTA),_xlfn.HSTACK("COUNTBLANK", _xleta.COUNTBLANK),_xlfn.HSTACK("COUNTIF", _xleta.COUNTIF),_xlfn.HSTACK("COUNTIFS", _xleta.COUNTIFS),_xlfn.HSTACK("COUPDAYBS", _xleta.COUPDAYBS),_xlfn.HSTACK("COUPDAYS", _xleta.COUPDAYS),_xlfn.HSTACK("COUPDAYSNC", _xleta.COUPDAYSNC),_xlfn.HSTACK("COUPNCD", _xleta.COUPNCD),_xlfn.HSTACK("COUPNUM", _xleta.COUPNUM),_xlfn.HSTACK("COUPPCD", _xleta.COUPPCD),_xlfn.HSTACK("COVAR", _xleta.COVAR),_xlfn.HSTACK("COVARIANCE.P", _xleta.COVARIANCE.P),_xlfn.HSTACK("COVARIANCE.S", _xleta.COVARIANCE.S),_xlfn.HSTACK("CRITBINOM", _xleta.CRITBINOM),_xlfn.HSTACK("CSC", _xleta.CSC),_xlfn.HSTACK("CSCH", _xleta.CSCH),_xlfn.HSTACK("CUBEKPIMEMBER", _xleta.CUBEKPIMEMBER),_xlfn.HSTACK("CUBEMEMBER", _xleta.CUBEMEMBER),_xlfn.HSTACK("CUBEMEMBERPROPERTY", _xleta.CUBEMEMBERPROPERTY),_xlfn.HSTACK("CUBERANKEDMEMBER", _xleta.CUBERANKEDMEMBER),_xlfn.HSTACK("CUBESET", _xleta.CUBESET),_xlfn.HSTACK("CUBESETCOUNT", _xleta.CUBESETCOUNT),_xlfn.HSTACK("CUBEVALUE", _xleta.CUBEVALUE),_xlfn.HSTACK("CUMIPMT", _xleta.CUMIPMT),_xlfn.HSTACK("CUMPRINC", _xleta.CUMPRINC)))</definedName>
     <definedName name="BUILTINS.D">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("DATE", _xleta.DATE),_xlfn.HSTACK("DATEDIF", _xleta.DATEDIF),_xlfn.HSTACK("DATEVALUE", _xleta.DATEVALUE),_xlfn.HSTACK("DAVERAGE", _xleta.DAVERAGE),_xlfn.HSTACK("DAY", _xleta.DAY),_xlfn.HSTACK("DAYS", _xleta.DAYS),_xlfn.HSTACK("DAYS360", _xleta.DAYS360),_xlfn.HSTACK("DB", _xleta.DB),_xlfn.HSTACK("DBCS", _xleta.DBCS),_xlfn.HSTACK("DCOUNT", _xleta.DCOUNT),_xlfn.HSTACK("DCOUNTA", _xleta.DCOUNTA),_xlfn.HSTACK("DDB", _xleta.DDB),_xlfn.HSTACK("DEC2BIN", _xleta.DEC2BIN),_xlfn.HSTACK("DEC2HEX", _xleta.DEC2HEX),_xlfn.HSTACK("DEC2OCT", _xleta.DEC2OCT),_xlfn.HSTACK("DECIMAL", _xleta.DECIMAL),_xlfn.HSTACK("DEGREES", _xleta.DEGREES),_xlfn.HSTACK("DELTA", _xleta.DELTA),_xlfn.HSTACK("DETECTLANGUAGE", _xleta.DETECTLANGUAGE),_xlfn.HSTACK("DEVSQ", _xleta.DEVSQ),_xlfn.HSTACK("DGET", _xleta.DGET),_xlfn.HSTACK("DISC", _xleta.DISC),_xlfn.HSTACK("DMAX", _xleta.DMAX),_xlfn.HSTACK("DMIN", _xleta.DMIN),_xlfn.HSTACK("DOLLAR", _xleta.DOLLAR),_xlfn.HSTACK("DOLLARDE", _xleta.DOLLARDE),_xlfn.HSTACK("DOLLARFR", _xleta.DOLLARFR),_xlfn.HSTACK("DPRODUCT", _xleta.DPRODUCT),_xlfn.HSTACK("DROP", _xleta.DROP),_xlfn.HSTACK("DSTDEV", _xleta.DSTDEV),_xlfn.HSTACK("DSTDEVP", _xleta.DSTDEVP),_xlfn.HSTACK("DSUM", _xleta.DSUM),_xlfn.HSTACK("DURATION", _xleta.DURATION),_xlfn.HSTACK("DVAR", _xleta.DVAR),_xlfn.HSTACK("DVARP", _xleta.DVARP)))</definedName>
     <definedName name="BUILTINS.E">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("EDATE", _xleta.EDATE),_xlfn.HSTACK("EFFECT", _xleta.EFFECT),_xlfn.HSTACK("ENCODEURL", _xleta.ENCODEURL),_xlfn.HSTACK("EOMONTH", _xleta.EOMONTH),_xlfn.HSTACK("ERF", _xleta.ERF),_xlfn.HSTACK("ERF.PRECISE", _xleta.ERF.PRECISE),_xlfn.HSTACK("ERFC", _xleta.ERFC),_xlfn.HSTACK("ERFC.PRECISE", _xleta.ERFC.PRECISE),_xlfn.HSTACK("ERROR.TYPE", _xleta.ERROR.TYPE),_xlfn.HSTACK("EVEN", _xleta.EVEN),_xlfn.HSTACK("EXACT", _xleta.EXACT),_xlfn.HSTACK("EXP", _xleta.EXP),_xlfn.HSTACK("EXPAND", _xleta.EXPAND),_xlfn.HSTACK("EXPON.DIST", _xleta.EXPON.DIST),_xlfn.HSTACK("EXPONDIST", _xleta.EXPONDIST)))</definedName>
-    <definedName name="BUILTINS.F">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("F.DIST", _xleta.F.DIST),_xlfn.HSTACK("F.DIST.RT", _xleta.F.DIST.RT),_xlfn.HSTACK("F.INV", _xleta.F.INV),_xlfn.HSTACK("F.INV.RT", _xleta.F.INV.RT),_xlfn.HSTACK("F.TEST", _xleta.F.TEST),_xlfn.HSTACK("FACT", _xleta.FACT),_xlfn.HSTACK("FACTDOUBLE", _xleta.FACTDOUBLE),_xlfn.HSTACK("FALSE", FALSE),_xlfn.HSTACK("FDIST", _xleta.FDIST),_xlfn.HSTACK("FIELDFUNCTION", _xleta.FIELDFUNCTION),_xlfn.HSTACK("FIELDVALUE", _xleta.FIELDVALUE),_xlfn.HSTACK("FILTER", _xleta.FILTER),_xlfn.HSTACK("FILTERXML", _xleta.FILTERXML),_xlfn.HSTACK("FIND", _xleta.FIND),_xlfn.HSTACK("FINDB", _xleta.FINDB),_xlfn.HSTACK("FINV", _xleta.FINV),_xlfn.HSTACK("FISHER", _xleta.FISHER),_xlfn.HSTACK("FISHERINV", _xleta.FISHERINV),_xlfn.HSTACK("FIXED", _xleta.FIXED),_xlfn.HSTACK("FLOOR", _xleta.FLOOR),_xlfn.HSTACK("FLOOR.MATH", _xleta.FLOOR.MATH),_xlfn.HSTACK("FLOOR.PRECISE", _xleta.FLOOR.PRECISE),_xlfn.HSTACK("FORECAST", _xleta.FORECAST),_xlfn.HSTACK("FORECAST.ETS", _xleta.FORECAST.ETS),_xlfn.HSTACK("FORECAST.ETS.CONFINT", _xleta.FORECAST.ETS.CONFINT),_xlfn.HSTACK("FORECAST.ETS.SEASONALITY", _xleta.FORECAST.ETS.SEASONALITY),_xlfn.HSTACK("FORECAST.ETS.STAT", _xleta.FORECAST.ETS.STAT),_xlfn.HSTACK("FORECAST.LINEAR", _xleta.FORECAST.LINEAR),_xlfn.HSTACK("FORMULATEXT", _xleta.FORMULATEXT),_xlfn.HSTACK("FREQUENCY", _xleta.FREQUENCY),_xlfn.HSTACK("FTEST", _xleta.FTEST),_xlfn.HSTACK("FV", _xleta.FV),_xlfn.HSTACK("FVSCHEDULE", _xleta.FVSCHEDULE)))</definedName>
+    <definedName name="BUILTINS.F">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("F.DIST", _xleta.F.DIST),_xlfn.HSTACK("F.DIST.RT", _xleta.F.DIST.RT),_xlfn.HSTACK("F.INV", _xleta.F.INV),_xlfn.HSTACK("F.INV.RT", _xleta.F.INV.RT),_xlfn.HSTACK("F.TEST", _xleta.F.TEST),_xlfn.HSTACK("FACT", _xleta.FACT),_xlfn.HSTACK("FACTDOUBLE", _xleta.FACTDOUBLE),_xlfn.HSTACK("FALSE", FALSE),_xlfn.HSTACK("FDIST", _xleta.FDIST),_xlfn.HSTACK("FIELDVALUE", _xleta.FIELDVALUE),_xlfn.HSTACK("FILTER", _xleta.FILTER),_xlfn.HSTACK("FILTERXML", _xleta.FILTERXML),_xlfn.HSTACK("FIND", _xleta.FIND),_xlfn.HSTACK("FINDB", _xleta.FINDB),_xlfn.HSTACK("FINV", _xleta.FINV),_xlfn.HSTACK("FISHER", _xleta.FISHER),_xlfn.HSTACK("FISHERINV", _xleta.FISHERINV),_xlfn.HSTACK("FIXED", _xleta.FIXED),_xlfn.HSTACK("FLOOR", _xleta.FLOOR),_xlfn.HSTACK("FLOOR.MATH", _xleta.FLOOR.MATH),_xlfn.HSTACK("FLOOR.PRECISE", _xleta.FLOOR.PRECISE),_xlfn.HSTACK("FORECAST", _xleta.FORECAST),_xlfn.HSTACK("FORECAST.ETS", _xleta.FORECAST.ETS),_xlfn.HSTACK("FORECAST.ETS.CONFINT", _xleta.FORECAST.ETS.CONFINT),_xlfn.HSTACK("FORECAST.ETS.SEASONALITY", _xleta.FORECAST.ETS.SEASONALITY),_xlfn.HSTACK("FORECAST.ETS.STAT", _xleta.FORECAST.ETS.STAT),_xlfn.HSTACK("FORECAST.LINEAR", _xleta.FORECAST.LINEAR),_xlfn.HSTACK("FORMULATEXT", _xleta.FORMULATEXT),_xlfn.HSTACK("FREQUENCY", _xleta.FREQUENCY),_xlfn.HSTACK("FTEST", _xleta.FTEST),_xlfn.HSTACK("FV", _xleta.FV),_xlfn.HSTACK("FVSCHEDULE", _xleta.FVSCHEDULE)))</definedName>
     <definedName name="BUILTINS.G">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("GAMMA", _xleta.GAMMA),_xlfn.HSTACK("GAMMA.DIST", _xleta.GAMMA.DIST),_xlfn.HSTACK("GAMMA.INV", _xleta.GAMMA.INV),_xlfn.HSTACK("GAMMADIST", _xleta.GAMMADIST),_xlfn.HSTACK("GAMMAINV", _xleta.GAMMAINV),_xlfn.HSTACK("GAMMALN", _xleta.GAMMALN),_xlfn.HSTACK("GAMMALN.PRECISE", _xleta.GAMMALN.PRECISE),_xlfn.HSTACK("GAUSS", _xleta.GAUSS),_xlfn.HSTACK("GCD", _xleta.GCD),_xlfn.HSTACK("GEOMEAN", _xleta.GEOMEAN),_xlfn.HSTACK("GESTEP", _xleta.GESTEP),_xlfn.HSTACK("GETPIVOTDATA", _xleta.GETPIVOTDATA),_xlfn.HSTACK("GROUPBY", _xleta.GROUPBY),_xlfn.HSTACK("GROWTH", _xleta.GROWTH)))</definedName>
     <definedName name="BUILTINS.H">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("HARMEAN", _xleta.HARMEAN),_xlfn.HSTACK("HEX2BIN", _xleta.HEX2BIN),_xlfn.HSTACK("HEX2DEC", _xleta.HEX2DEC),_xlfn.HSTACK("HEX2OCT", _xleta.HEX2OCT),_xlfn.HSTACK("HLOOKUP", _xleta.HLOOKUP),_xlfn.HSTACK("HOUR", _xleta.HOUR),_xlfn.HSTACK("HSTACK", _xleta.HSTACK),_xlfn.HSTACK("HYPERLINK", _xleta.HYPERLINK),_xlfn.HSTACK("HYPGEOM.DIST", _xleta.HYPGEOM.DIST),_xlfn.HSTACK("HYPGEOMDIST", _xleta.HYPGEOMDIST)))</definedName>
     <definedName name="BUILTINS.I">_xlfn.LAMBDA(_xlfn.VSTACK(_xlfn.HSTACK("IF", _xleta.IF),_xlfn.HSTACK("IFERROR", _xleta.IFERROR),_xlfn.HSTACK("IFNA", _xleta.IFNA),_xlfn.HSTACK("IFS", _xleta.IFS),_xlfn.HSTACK("IMABS", _xleta.IMABS),_xlfn.HSTACK("IMAGE", _xleta.IMAGE),_xlfn.HSTACK("IMAGINARY", _xleta.IMAGINARY),_xlfn.HSTACK("IMARGUMENT", _xleta.IMARGUMENT),_xlfn.HSTACK("IMCONJUGATE", _xleta.IMCONJUGATE),_xlfn.HSTACK("IMCOS", _xleta.IMCOS),_xlfn.HSTACK("IMCOSH", _xleta.IMCOSH),_xlfn.HSTACK("IMCOT", _xleta.IMCOT),_xlfn.HSTACK("IMCSC", _xleta.IMCSC),_xlfn.HSTACK("IMCSCH", _xleta.IMCSCH),_xlfn.HSTACK("IMDIV", _xleta.IMDIV),_xlfn.HSTACK("IMEXP", _xleta.IMEXP),_xlfn.HSTACK("IMLN", _xleta.IMLN),_xlfn.HSTACK("IMLOG10", _xleta.IMLOG10),_xlfn.HSTACK("IMLOG2", _xleta.IMLOG2),_xlfn.HSTACK("IMPOWER", _xleta.IMPOWER),_xlfn.HSTACK("IMPRODUCT", _xleta.IMPRODUCT),_xlfn.HSTACK("IMREAL", _xleta.IMREAL),_xlfn.HSTACK("IMSEC", _xleta.IMSEC),_xlfn.HSTACK("IMSECH", _xleta.IMSECH),_xlfn.HSTACK("IMSIN", _xleta.IMSIN),_xlfn.HSTACK("IMSINH", _xleta.IMSINH),_xlfn.HSTACK("IMSQRT", _xleta.IMSQRT),_xlfn.HSTACK("IMSUB", _xleta.IMSUB),_xlfn.HSTACK("IMSUM", _xleta.IMSUM),_xlfn.HSTACK("IMTAN", _xleta.IMTAN),_xlfn.HSTACK("INDEX", _xleta.INDEX),_xlfn.HSTACK("INDIRECT", _xleta.INDIRECT),_xlfn.HSTACK("INFO", _xleta.INFO),_xlfn.HSTACK("INT", _xleta.INT),_xlfn.HSTACK("INTERCEPT", _xleta.INTERCEPT),_xlfn.HSTACK("INTRATE", _xleta.INTRATE),_xlfn.HSTACK("IPMT", _xleta.IPMT),_xlfn.HSTACK("IRR", _xleta.IRR),_xlfn.HSTACK("ISBLANK", _xleta.ISBLANK),_xlfn.HSTACK("ISERR", _xleta.ISERR),_xlfn.HSTACK("ISERROR", _xleta.ISERROR),_xlfn.HSTACK("ISEVEN", _xleta.ISEVEN),_xlfn.HSTACK("ISFORMULA", _xleta.ISFORMULA),_xlfn.HSTACK("ISLOGICAL", _xleta.ISLOGICAL),_xlfn.HSTACK("ISNA", _xleta.ISNA),_xlfn.HSTACK("ISNONTEXT", _xleta.ISNONTEXT),_xlfn.HSTACK("ISNUMBER", _xleta.ISNUMBER),_xlfn.HSTACK("ISODD", _xleta.ISODD),_xlfn.HSTACK("ISOMITTED", _xleta.ISOMITTED),_xlfn.HSTACK("ISOWEEKNUM", _xleta.ISOWEEKNUM),_xlfn.HSTACK("ISPMT", _xleta.ISPMT),_xlfn.HSTACK("ISREF", _xleta.ISREF),_xlfn.HSTACK("ISTEXT", _xleta.ISTEXT)))</definedName>
@@ -140,6 +142,7 @@
     <definedName name="TEXTBETWEEN">_xlfn.LAMBDA(_xlpm.source_text,_xlpm.first_boundary,_xlpm.second_boundary,_xlfn.LET(_xlpm.text_after_first_boundary,RIGHT(_xlpm.source_text,DIFFERENCE(LEN(_xlpm.source_text),DECREMENT(SUM(FIND(_xlpm.first_boundary,_xlpm.source_text),LEN(_xlpm.first_boundary))))),LEFT(_xlpm.text_after_first_boundary,DECREMENT(FIND(_xlpm.second_boundary,_xlpm.text_after_first_boundary)))))</definedName>
     <definedName name="TEXTTOCOLUMNS">_xlfn.LAMBDA(_xlpm.text,_xlpm.delimiter,_xlfn.TEXTSPLIT(_xlpm.text,_xlpm.delimiter))</definedName>
     <definedName name="TEXTTOROWS">_xlfn.LAMBDA(_xlpm.text,_xlpm.delimiter,TRANSPOSE(_xlfn.TEXTSPLIT(_xlpm.text,_xlpm.delimiter)))</definedName>
+    <definedName name="TODO">_xlfn.LAMBDA(_xlpm.description,_xlpm.description)</definedName>
     <definedName name="TRIMALL">_xlfn.LAMBDA(_xlpm.range,_xlfn.MAKEARRAY(ROWS(_xlpm.range),COLUMNS(_xlpm.range),_xlfn.LAMBDA(_xlpm.row,_xlpm.col,TRIM(INDEX(_xlpm.range,_xlpm.row,_xlpm.col)))))</definedName>
     <definedName name="TRIMSPLIT">_xlfn.LAMBDA(_xlpm.source_text,_xlpm.split_at,_xlop.display_vertically,_xlfn.LET(_xlpm.result,TRIMALL(_xlfn.TEXTSPLIT(_xlpm.source_text,_xlpm.split_at)),IF(DEFAULT(_xlpm.display_vertically,FALSE),TRANSPOSE(_xlpm.result),_xlpm.result)))</definedName>
     <definedName name="TYPESTRING">_xlfn.LAMBDA(_xlpm.input,_xlop.recursive,_xlfn.SWITCH(TYPE(_xlpm.input),1,"Number",2,"String",4,"Boolean",16,"Error",64,IF(DEFAULT(_xlpm.recursive,FALSE),_xlfn.MAP(_xlpm.input,_xlfn.LAMBDA(_xlpm.each,TYPESTRING(_xlpm.each))),"Range"),128,"Function",OTHERWISE,"Unknown"))</definedName>
@@ -670,7 +673,7 @@
       </c>
       <c r="C4" s="3" t="str" cm="1">
         <f t="array" aca="1" ref="C4:C13" ca="1">FLIPCOIN(10)</f>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -697,7 +700,7 @@
       </c>
       <c r="C6" s="3" t="str">
         <f ca="1"/>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -720,7 +723,7 @@
       </c>
       <c r="C8" s="3" t="str">
         <f ca="1"/>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
       <c r="E8" t="s">
         <v>7</v>
@@ -733,7 +736,7 @@
       </c>
       <c r="C9" s="3" t="str">
         <f ca="1"/>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
       <c r="E9" t="s">
         <v>8</v>
@@ -750,7 +753,7 @@
       </c>
       <c r="C10" s="3" t="str">
         <f ca="1"/>
-        <v>Heads</v>
+        <v>Tails</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -760,7 +763,7 @@
       </c>
       <c r="C11" s="3" t="str">
         <f ca="1"/>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
       <c r="E11" t="s">
         <v>10</v>
@@ -777,7 +780,7 @@
       </c>
       <c r="C12" s="3" t="str">
         <f ca="1"/>
-        <v>Tails</v>
+        <v>Heads</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>